<commit_message>
Cleaned Up Design Documents
Cleaned Up Design Documents
</commit_message>
<xml_diff>
--- a/T41_V012_Files/T41_V012_Design_Documents/T41_V12.6_I2C_Assignments.xlsx
+++ b/T41_V012_Files/T41_V012_Design_Documents/T41_V12.6_I2C_Assignments.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dad\Documents\GitHub\T41\T41_V012_Files\T41_V012_Design_Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D19CE9-72FB-489B-A75E-9AAD5949F93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48C04B87-7219-47FB-AE81-B9FEE998E55A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="231">
   <si>
     <t>I2C Addresses For The T41 V012.6</t>
   </si>
@@ -89,9 +89,6 @@
     <t>Wire</t>
   </si>
   <si>
-    <t>19-20</t>
-  </si>
-  <si>
     <t>RFControl</t>
   </si>
   <si>
@@ -122,9 +119,6 @@
     <t>Display</t>
   </si>
   <si>
-    <t>0x40/0x38</t>
-  </si>
-  <si>
     <t>Touch Screen Controller</t>
   </si>
   <si>
@@ -168,9 +162,6 @@
   </si>
   <si>
     <t>Si5351a Frequency Control - Primary Receiver and Transmitter</t>
-  </si>
-  <si>
-    <t>0x61/0x6F</t>
   </si>
   <si>
     <t>Si5351a Frequency Control - Second Receiver</t>
@@ -476,15 +467,9 @@
     </r>
   </si>
   <si>
-    <t>0x60/ 0x61/ 0x6F</t>
-  </si>
-  <si>
     <t>Si5351a</t>
   </si>
   <si>
-    <t xml:space="preserve"> Frequency Control - Primary Receiver and Transmitter (0x60), Second Receiver (0x61 or 0x6F)</t>
-  </si>
-  <si>
     <t>RC-0.5 dB Receive Signal Reduction ["1"=On, "0"= Off]</t>
   </si>
   <si>
@@ -506,9 +491,6 @@
     <t>N/C</t>
   </si>
   <si>
-    <t>MF or HF Select - "1"=MF, "0"=HF</t>
-  </si>
-  <si>
     <t>TC-0.5 dB Transmit Power Reduction ["1"=On, "0"= Off]</t>
   </si>
   <si>
@@ -533,9 +515,6 @@
     <t>BPF Board - I2C Addresses</t>
   </si>
   <si>
-    <t>BPF #1</t>
-  </si>
-  <si>
     <t>High = 12M</t>
   </si>
   <si>
@@ -611,9 +590,6 @@
     <t>High = 15M</t>
   </si>
   <si>
-    <t>BPF #2</t>
-  </si>
-  <si>
     <t>LPF Board - I2C Addresses</t>
   </si>
   <si>
@@ -674,12 +650,6 @@
     <t>MCP23017 for Band LPF Selection 160M-6M+Bypass, 1-4 Antenna Selection, XVTR Selection, 100W Module Selection, BPF TX &amp; RX Selection.</t>
   </si>
   <si>
-    <t>0x27/ 0x23</t>
-  </si>
-  <si>
-    <t>111/ 011</t>
-  </si>
-  <si>
     <t>ATU Module - I2C Addresses</t>
   </si>
   <si>
@@ -747,13 +717,43 @@
   </si>
   <si>
     <t>C8 - 2000pF</t>
+  </si>
+  <si>
+    <t>18-19</t>
+  </si>
+  <si>
+    <t>BPF FOR RX  #1</t>
+  </si>
+  <si>
+    <t>BPF FOR RX #2</t>
+  </si>
+  <si>
+    <t>RX #1</t>
+  </si>
+  <si>
+    <t>RX #2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Frequency Control - Receiver and Transmitter (0x60)</t>
+  </si>
+  <si>
+    <t>DEVICE</t>
+  </si>
+  <si>
+    <t>0x61 or 0x6F</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Frequency Control - Second Receiver (0x61 or 0x6F)</t>
+  </si>
+  <si>
+    <t>0x40 or 0x38</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -844,6 +844,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -871,7 +877,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -931,6 +937,12 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1362,10 +1374,10 @@
         <v>17</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>19</v>
       </c>
       <c r="E6" s="1">
         <v>1</v>
@@ -1374,10 +1386,10 @@
         <v>3</v>
       </c>
       <c r="G6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="M6" s="10" t="s">
         <v>15</v>
@@ -1385,13 +1397,13 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="9" t="s">
         <v>23</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>24</v>
       </c>
       <c r="E7" s="1">
         <v>5</v>
@@ -1405,13 +1417,13 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="9" t="s">
         <v>26</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>27</v>
       </c>
       <c r="E8" s="1">
         <v>7</v>
@@ -1436,13 +1448,13 @@
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E10" s="1">
         <v>7</v>
@@ -1451,13 +1463,13 @@
         <v>5</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>29</v>
+        <v>230</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>15</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="M10" s="10"/>
     </row>
@@ -1474,13 +1486,13 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E12" s="1">
         <v>5</v>
@@ -1489,13 +1501,13 @@
         <v>7</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="H12" s="12" t="s">
         <v>15</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="M12" s="10" t="s">
         <v>15</v>
@@ -1503,17 +1515,17 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D13" s="9"/>
       <c r="G13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="M13" s="10"/>
     </row>
@@ -1521,13 +1533,13 @@
       <c r="A14" s="5"/>
       <c r="D14" s="9"/>
       <c r="G14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I14" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="M14" s="10"/>
     </row>
@@ -1544,13 +1556,13 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E16" s="1">
         <v>1</v>
@@ -1559,43 +1571,43 @@
         <v>3</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D17" s="9"/>
       <c r="G17" s="1" t="s">
-        <v>45</v>
+        <v>228</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D18" s="9"/>
       <c r="G18" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H18" s="1">
         <v>111</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D19" s="9"/>
       <c r="G19" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:9" s="7" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1610,13 +1622,13 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E21" s="1">
         <v>7</v>
@@ -1625,26 +1637,26 @@
         <v>5</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" s="5"/>
       <c r="D22" s="9"/>
       <c r="G22" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="H22" s="1">
         <v>110</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:9" s="7" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1659,13 +1671,13 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E24" s="1">
         <v>7</v>
@@ -1674,27 +1686,27 @@
         <v>5</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
     </row>
     <row r="26" spans="1:9" s="7" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1709,13 +1721,13 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E27" s="1">
         <v>1</v>
@@ -1724,10 +1736,10 @@
         <v>3</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:9" s="7" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1742,13 +1754,13 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E29" s="1">
         <v>7</v>
@@ -1757,24 +1769,24 @@
         <v>5</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:9" s="7" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1789,13 +1801,13 @@
     </row>
     <row r="32" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E32" s="1">
         <v>7</v>
@@ -1804,27 +1816,27 @@
         <v>5</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H32" s="26" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="H33" s="26" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
     </row>
     <row r="34" spans="1:9" s="7" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1839,7 +1851,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" s="14" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1864,7 +1876,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="16" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.4">
@@ -1890,10 +1902,10 @@
         <v>8</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.4">
@@ -1921,10 +1933,10 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A6" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C6" s="18">
         <v>7</v>
@@ -1933,24 +1945,24 @@
         <v>5</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H6" s="18" t="s">
         <v>15</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A7" s="18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" s="18">
         <v>7</v>
@@ -1959,18 +1971,18 @@
         <v>5</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A9" s="20" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1996,7 +2008,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="16" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
@@ -2025,10 +2037,10 @@
         <v>8</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I3" s="21" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2065,10 +2077,10 @@
     </row>
     <row r="6" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C6" s="1">
         <v>5</v>
@@ -2077,16 +2089,16 @@
         <v>7</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2095,19 +2107,19 @@
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2116,10 +2128,10 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2131,10 +2143,10 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2146,10 +2158,10 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2161,10 +2173,10 @@
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2176,10 +2188,10 @@
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2191,10 +2203,10 @@
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2206,10 +2218,10 @@
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2221,10 +2233,10 @@
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2236,10 +2248,10 @@
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2251,10 +2263,10 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2266,10 +2278,10 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2281,10 +2293,10 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2296,10 +2308,10 @@
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2311,10 +2323,10 @@
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2326,10 +2338,10 @@
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="23" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2338,19 +2350,19 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2362,10 +2374,10 @@
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2383,10 +2395,10 @@
         <v>15</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="26" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2398,10 +2410,10 @@
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="27" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2413,10 +2425,10 @@
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2428,10 +2440,10 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="29" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2447,82 +2459,82 @@
         <v>15</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="H30" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="H31" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="H32" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="8:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="H33" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34" spans="8:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="H34" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" spans="8:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="H35" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="36" spans="8:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="H36" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="37" spans="8:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="H37" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="38" spans="8:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="H38" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2533,7 +2545,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:AMJ25"/>
+  <dimension ref="A1:AMJ44"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="15"/>
@@ -2550,7 +2562,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="16" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.4">
@@ -2567,7 +2579,7 @@
         <v>6</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>8</v>
@@ -2576,10 +2588,10 @@
         <v>8</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.4">
@@ -2617,38 +2629,43 @@
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.4">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="1">
+      <c r="B7" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="1">
         <v>1</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D7" s="1">
         <v>3</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" s="15" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
-      <c r="A7" s="1"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="2"/>
+      <c r="E7" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A8" s="1"/>
@@ -2656,19 +2673,19 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>206</v>
+        <v>44</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>207</v>
+        <v>85</v>
+      </c>
+      <c r="G8" s="1">
+        <v>111</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.4">
@@ -2683,127 +2700,317 @@
         <v>15</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.4">
       <c r="H10" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.4">
       <c r="H11" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I11" s="15" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.4">
       <c r="H12" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.4">
       <c r="H13" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.4">
       <c r="H14" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.4">
       <c r="H15" s="2" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.4">
       <c r="H16" s="15" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I16" s="15" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="H17" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="H18" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="I18" s="15" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="H19" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="I19" s="15" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="H20" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="I20" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="H21" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="I21" s="15" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="H22" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="I22" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="H23" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="I23" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A25" s="27" t="s">
+        <v>225</v>
+      </c>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="2"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A26" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="1">
+        <v>1</v>
+      </c>
+      <c r="D26" s="1">
+        <v>3</v>
+      </c>
+      <c r="E26" s="28" t="s">
+        <v>228</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="G26" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="I26" s="15" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A27" s="1"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F27" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="G27" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I27" s="15" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A28" s="1"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I28" s="15" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="H29" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="I29" s="15" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="H30" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I30" s="15" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="H31" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I31" s="15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="H32" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="I32" s="15" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.4">
+      <c r="H33" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I33" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.4">
+      <c r="H34" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="I34" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.4">
+      <c r="H35" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="I35" s="15" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.4">
+      <c r="H36" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="I36" s="15" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.4">
+      <c r="H37" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="I37" s="15" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.4">
+      <c r="H38" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="I38" s="15" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.4">
+      <c r="H39" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="I39" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.4">
+      <c r="H40" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="I40" s="15" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.4">
+      <c r="H41" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="I41" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.4">
+      <c r="H42" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="I42" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.4">
+      <c r="B44" s="22" t="s">
         <v>151</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="H17" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="I17" s="15" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="H18" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="I18" s="15" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="H19" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="I19" s="15" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="H20" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="I20" s="15" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="H21" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="I21" s="15" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="H22" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="I22" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="H23" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="I23" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B25" s="22" t="s">
-        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -2836,7 +3043,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="16" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:26" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -2862,10 +3069,10 @@
         <v>8</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -2953,7 +3160,7 @@
     </row>
     <row r="6" spans="1:26" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
-        <v>159</v>
+        <v>222</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -2982,10 +3189,10 @@
     </row>
     <row r="7" spans="1:26" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" s="1">
         <v>7</v>
@@ -2994,70 +3201,70 @@
         <v>5</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="L7" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>91</v>
-      </c>
       <c r="M7" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="X7" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="Y7" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="Z7" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:26" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -3066,10 +3273,10 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
@@ -3096,13 +3303,13 @@
       <c r="D9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="K9" s="1">
         <v>0</v>
@@ -3162,13 +3369,13 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="K10" s="1">
         <v>0</v>
@@ -3228,13 +3435,13 @@
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="K11" s="1">
         <v>0</v>
@@ -3294,13 +3501,13 @@
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="K12" s="1">
         <v>0</v>
@@ -3360,13 +3567,13 @@
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="K13" s="1">
         <v>0</v>
@@ -3426,13 +3633,13 @@
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="K14" s="1">
         <v>0</v>
@@ -3492,13 +3699,13 @@
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="K15" s="1">
         <v>0</v>
@@ -3558,13 +3765,13 @@
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="K16" s="1">
         <v>0</v>
@@ -3624,13 +3831,13 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="K17" s="1">
         <v>1</v>
@@ -3690,13 +3897,13 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="K18" s="1">
         <v>0</v>
@@ -3756,13 +3963,13 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="K19" s="1">
         <v>0</v>
@@ -3822,13 +4029,13 @@
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="K20" s="1">
         <v>0</v>
@@ -3888,10 +4095,10 @@
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
@@ -3920,10 +4127,10 @@
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
@@ -3945,15 +4152,15 @@
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A24" s="25" t="s">
-        <v>185</v>
+        <v>223</v>
       </c>
     </row>
     <row r="25" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C25" s="1">
         <v>7</v>
@@ -3962,70 +4169,70 @@
         <v>5</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F25" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="L25" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="G25" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="K25" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="L25" s="1" t="s">
-        <v>91</v>
-      </c>
       <c r="M25" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="Q25" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="S25" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="T25" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="U25" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="V25" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="W25" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="X25" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="Y25" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="Z25" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="26" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
@@ -4037,10 +4244,10 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
@@ -4069,13 +4276,13 @@
       <c r="F27" s="2"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="K27" s="1">
         <v>0</v>
@@ -4135,13 +4342,13 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="K28" s="1">
         <v>0</v>
@@ -4201,13 +4408,13 @@
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="K29" s="1">
         <v>0</v>
@@ -4267,13 +4474,13 @@
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="K30" s="1">
         <v>0</v>
@@ -4333,13 +4540,13 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="K31" s="1">
         <v>0</v>
@@ -4399,13 +4606,13 @@
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="K32" s="1">
         <v>0</v>
@@ -4465,13 +4672,13 @@
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="K33" s="1">
         <v>0</v>
@@ -4531,13 +4738,13 @@
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="K34" s="1">
         <v>0</v>
@@ -4597,13 +4804,13 @@
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="K35" s="1">
         <v>1</v>
@@ -4663,13 +4870,13 @@
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="K36" s="1">
         <v>0</v>
@@ -4729,13 +4936,13 @@
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="K37" s="1">
         <v>0</v>
@@ -4795,13 +5002,13 @@
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="K38" s="1">
         <v>0</v>
@@ -4861,10 +5068,10 @@
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
@@ -4893,10 +5100,10 @@
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="J40" s="1"/>
       <c r="K40" s="1"/>
@@ -4944,7 +5151,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="16" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:14" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -4970,10 +5177,10 @@
         <v>8</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -5025,10 +5232,10 @@
     </row>
     <row r="6" spans="1:14" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C6" s="1">
         <v>7</v>
@@ -5037,34 +5244,34 @@
         <v>5</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="L6" s="24" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:14" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5073,10 +5280,10 @@
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="H7" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
@@ -5091,13 +5298,13 @@
       <c r="D8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="K8" s="1">
         <v>0</v>
@@ -5121,13 +5328,13 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="K9" s="1">
         <v>0</v>
@@ -5151,13 +5358,13 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="K10" s="1">
         <v>0</v>
@@ -5181,13 +5388,13 @@
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="K11" s="1">
         <v>0</v>
@@ -5211,13 +5418,13 @@
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="K12" s="1">
         <v>0</v>
@@ -5241,13 +5448,13 @@
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="K13" s="1">
         <v>0</v>
@@ -5271,13 +5478,13 @@
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="K14" s="1">
         <v>0</v>
@@ -5301,13 +5508,13 @@
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="K15" s="1">
         <v>0</v>
@@ -5331,13 +5538,13 @@
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="K16" s="1">
         <v>1</v>
@@ -5361,13 +5568,13 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="K17" s="1">
         <v>1</v>
@@ -5391,13 +5598,13 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="K18" s="1">
         <v>1</v>
@@ -5421,13 +5628,13 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="K19" s="1">
         <v>1</v>
@@ -5451,10 +5658,10 @@
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
@@ -5471,10 +5678,10 @@
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
@@ -5509,19 +5716,19 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
@@ -5544,10 +5751,10 @@
         <v>15</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
@@ -5562,10 +5769,10 @@
       <c r="D25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
@@ -5582,10 +5789,10 @@
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
@@ -5651,7 +5858,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="16" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5677,10 +5884,10 @@
         <v>8</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5717,10 +5924,10 @@
     </row>
     <row r="6" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C6" s="1">
         <v>7</v>
@@ -5729,19 +5936,19 @@
         <v>5</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G6" s="26" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
     </row>
     <row r="7" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5750,10 +5957,10 @@
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="H7" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5763,10 +5970,10 @@
       <c r="D8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5778,10 +5985,10 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5793,10 +6000,10 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5808,10 +6015,10 @@
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
     </row>
     <row r="12" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5823,10 +6030,10 @@
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5838,10 +6045,10 @@
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
     </row>
     <row r="14" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5853,10 +6060,10 @@
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
     </row>
     <row r="15" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5868,10 +6075,10 @@
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
     </row>
     <row r="16" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5883,10 +6090,10 @@
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
     </row>
     <row r="17" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5898,10 +6105,10 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
     </row>
     <row r="18" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5913,10 +6120,10 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
     </row>
     <row r="19" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5928,10 +6135,10 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5943,10 +6150,10 @@
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
     </row>
     <row r="21" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5958,10 +6165,10 @@
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
     </row>
     <row r="22" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -5986,19 +6193,19 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
     </row>
     <row r="24" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -6016,10 +6223,10 @@
         <v>15</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
     </row>
     <row r="25" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -6029,10 +6236,10 @@
       <c r="D25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
     </row>
     <row r="26" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -6044,10 +6251,10 @@
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="27" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -6059,10 +6266,10 @@
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="28" spans="1:9" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
@@ -6078,26 +6285,26 @@
         <v>15</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="H29" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="H30" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -6118,7 +6325,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="16" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.4">
@@ -6144,10 +6351,10 @@
         <v>8</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.4">
@@ -6175,7 +6382,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.4">
       <c r="B6" s="15" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -6196,7 +6403,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="16" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.4">
@@ -6222,10 +6429,10 @@
         <v>8</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.4">
@@ -6253,7 +6460,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.4">
       <c r="B6" s="15" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>